<commit_message>
feat(coach): add some more instruction in posture: maintain neu
</commit_message>
<xml_diff>
--- a/DASHBOARD/fitness_dashboard.xlsx
+++ b/DASHBOARD/fitness_dashboard.xlsx
@@ -780,8 +780,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H9" headerRowCount="1">
-  <autoFilter ref="A1:H9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H8" headerRowCount="1">
+  <autoFilter ref="A1:H8"/>
   <tableColumns count="8">
     <tableColumn id="1" name="workout_id"/>
     <tableColumn id="2" name="date"/>
@@ -797,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N127" headerRowCount="1">
-  <autoFilter ref="A1:N127"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N126" headerRowCount="1">
+  <autoFilter ref="A1:N126"/>
   <tableColumns count="14">
     <tableColumn id="1" name="set_id"/>
     <tableColumn id="2" name="workout_id"/>
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1867,44 +1867,6 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>W-20261012-01</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>Pull</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Pull Workout</t>
-        </is>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>60</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="G9" s="19" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="H9" s="19" t="inlineStr">
-        <is>
-          <t>Update log and everything in just update commit to the app we have to show next pull session</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1919,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N127"/>
+  <dimension ref="A1:N126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1935,7 +1897,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="96" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7785,58 +7747,6 @@
         <v>0</v>
       </c>
       <c r="N126" s="19" t="n"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="19" t="inlineStr">
-        <is>
-          <t>S-20261012-01-01</t>
-        </is>
-      </c>
-      <c r="B127" s="19" t="inlineStr">
-        <is>
-          <t>W-20261012-01</t>
-        </is>
-      </c>
-      <c r="C127" s="19" t="inlineStr">
-        <is>
-          <t>PULL_UP</t>
-        </is>
-      </c>
-      <c r="D127" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E127" s="19" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F127" s="19" t="n"/>
-      <c r="G127" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H127" s="19" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="I127" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="J127" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K127" s="19" t="n"/>
-      <c r="L127" s="19" t="n">
-        <v>90</v>
-      </c>
-      <c r="M127" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N127" s="19" t="inlineStr">
-        <is>
-          <t>Update log and everything in just update commit to the app we have to show next pull session</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(workout): ingest Leg & Core session W-20261013-01 and prescribe Push B
</commit_message>
<xml_diff>
--- a/DASHBOARD/fitness_dashboard.xlsx
+++ b/DASHBOARD/fitness_dashboard.xlsx
@@ -780,8 +780,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H8" headerRowCount="1">
-  <autoFilter ref="A1:H8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H9" headerRowCount="1">
+  <autoFilter ref="A1:H9"/>
   <tableColumns count="8">
     <tableColumn id="1" name="workout_id"/>
     <tableColumn id="2" name="date"/>
@@ -797,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N126" headerRowCount="1">
-  <autoFilter ref="A1:N126"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N147" headerRowCount="1">
+  <autoFilter ref="A1:N147"/>
   <tableColumns count="14">
     <tableColumn id="1" name="set_id"/>
     <tableColumn id="2" name="workout_id"/>
@@ -820,8 +820,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I32" headerRowCount="1">
-  <autoFilter ref="A1:I32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I34" headerRowCount="1">
+  <autoFilter ref="A1:I34"/>
   <tableColumns count="9">
     <tableColumn id="1" name="exercise_id"/>
     <tableColumn id="2" name="exercise_name"/>
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1560,7 +1560,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="143" customWidth="1" min="8" max="8"/>
+    <col width="595" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1864,6 +1864,74 @@
       <c r="H8" s="19" t="inlineStr">
         <is>
           <t>Duration 63m 10s. Full workout report recovered. Efficient session, front raises removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>LEGS</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Day 3: Legs &amp; Core</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>37</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Workout
+2026-10-13 22:26
+Duration: 37m 42s
+Leg Press
+Set 1: 12 reps x 18.0 kg
+Set 2: 12 reps x 45.0 kg
+Set 3: 12 reps x 45.0 kg
+Set 4: 12 reps x 45.0 kg
+Leg Extension
+Set 1: 12 reps x 5.0 kg
+Set 2: 12 reps x 10.0 kg
+Set 3: 12 reps x 7.5 kg
+Set 4: 12 reps x 7.5 kg
+Lying Leg Curl
+Set 1: 12 reps x 5.0 kg
+Set 2: 10 reps x 5.0 kg
+Set 3: 8 reps x 5.0 kg
+Standing Calf Raise
+Set 1: 12 reps x 80.0 kg
+Set 2: 12 reps x 80.0 kg
+Set 3: 12 reps x 80.0 kg
+Crunch
+Set 1: 12 reps
+Set 2: 12 reps
+Set 3: 12 reps
+Dead Bug
+Set 1: 12 reps
+Set 2: 12 reps
+Set 3: 12 reps
+Lying Leg Raises
+Set 1: 12 reps x 0.0 kg</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N126"/>
+  <dimension ref="A1:N147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1897,7 +1965,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="27" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7747,6 +7815,1098 @@
         <v>0</v>
       </c>
       <c r="N126" s="19" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-01</t>
+        </is>
+      </c>
+      <c r="B127" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C127" s="19" t="inlineStr">
+        <is>
+          <t>LEG_PRESS</t>
+        </is>
+      </c>
+      <c r="D127" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E127" s="19" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="F127" s="19" t="n"/>
+      <c r="G127" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="H127" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I127" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J127" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K127" s="19" t="n"/>
+      <c r="L127" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M127" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 18.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-02</t>
+        </is>
+      </c>
+      <c r="B128" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C128" s="19" t="inlineStr">
+        <is>
+          <t>LEG_PRESS</t>
+        </is>
+      </c>
+      <c r="D128" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E128" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F128" s="19" t="n"/>
+      <c r="G128" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H128" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I128" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J128" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K128" s="19" t="n"/>
+      <c r="L128" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M128" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 45.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-03</t>
+        </is>
+      </c>
+      <c r="B129" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C129" s="19" t="inlineStr">
+        <is>
+          <t>LEG_PRESS</t>
+        </is>
+      </c>
+      <c r="D129" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E129" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F129" s="19" t="n"/>
+      <c r="G129" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H129" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I129" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J129" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K129" s="19" t="n"/>
+      <c r="L129" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M129" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 12 reps x 45.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-04</t>
+        </is>
+      </c>
+      <c r="B130" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C130" s="19" t="inlineStr">
+        <is>
+          <t>LEG_PRESS</t>
+        </is>
+      </c>
+      <c r="D130" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E130" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F130" s="19" t="n"/>
+      <c r="G130" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H130" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I130" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J130" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K130" s="19" t="n"/>
+      <c r="L130" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M130" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N130" s="19" t="inlineStr">
+        <is>
+          <t>Set 4: 12 reps x 45.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-05</t>
+        </is>
+      </c>
+      <c r="B131" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C131" s="19" t="inlineStr">
+        <is>
+          <t>LEG_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D131" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E131" s="19" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="F131" s="19" t="n"/>
+      <c r="G131" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H131" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I131" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J131" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K131" s="19" t="n"/>
+      <c r="L131" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M131" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-06</t>
+        </is>
+      </c>
+      <c r="B132" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C132" s="19" t="inlineStr">
+        <is>
+          <t>LEG_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D132" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E132" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F132" s="19" t="n"/>
+      <c r="G132" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H132" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I132" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J132" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K132" s="19" t="n"/>
+      <c r="L132" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M132" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 10.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-07</t>
+        </is>
+      </c>
+      <c r="B133" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C133" s="19" t="inlineStr">
+        <is>
+          <t>LEG_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D133" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E133" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F133" s="19" t="n"/>
+      <c r="G133" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H133" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I133" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J133" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K133" s="19" t="n"/>
+      <c r="L133" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M133" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 12 reps x 7.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-08</t>
+        </is>
+      </c>
+      <c r="B134" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C134" s="19" t="inlineStr">
+        <is>
+          <t>LEG_EXTENSION</t>
+        </is>
+      </c>
+      <c r="D134" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E134" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F134" s="19" t="n"/>
+      <c r="G134" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H134" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I134" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J134" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K134" s="19" t="n"/>
+      <c r="L134" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M134" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" s="19" t="inlineStr">
+        <is>
+          <t>Set 4: 12 reps x 7.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-09</t>
+        </is>
+      </c>
+      <c r="B135" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C135" s="19" t="inlineStr">
+        <is>
+          <t>LEG_CURL</t>
+        </is>
+      </c>
+      <c r="D135" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E135" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F135" s="19" t="n"/>
+      <c r="G135" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H135" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I135" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J135" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K135" s="19" t="n"/>
+      <c r="L135" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M135" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-10</t>
+        </is>
+      </c>
+      <c r="B136" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C136" s="19" t="inlineStr">
+        <is>
+          <t>LEG_CURL</t>
+        </is>
+      </c>
+      <c r="D136" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E136" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F136" s="19" t="n"/>
+      <c r="G136" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H136" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I136" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J136" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K136" s="19" t="n"/>
+      <c r="L136" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M136" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N136" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 10 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-11</t>
+        </is>
+      </c>
+      <c r="B137" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C137" s="19" t="inlineStr">
+        <is>
+          <t>LEG_CURL</t>
+        </is>
+      </c>
+      <c r="D137" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E137" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F137" s="19" t="n"/>
+      <c r="G137" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H137" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I137" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J137" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K137" s="19" t="n"/>
+      <c r="L137" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M137" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 8 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-12</t>
+        </is>
+      </c>
+      <c r="B138" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C138" s="19" t="inlineStr">
+        <is>
+          <t>CALF_RAISE</t>
+        </is>
+      </c>
+      <c r="D138" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E138" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F138" s="19" t="n"/>
+      <c r="G138" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="H138" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I138" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J138" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K138" s="19" t="n"/>
+      <c r="L138" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M138" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 80.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-13</t>
+        </is>
+      </c>
+      <c r="B139" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C139" s="19" t="inlineStr">
+        <is>
+          <t>CALF_RAISE</t>
+        </is>
+      </c>
+      <c r="D139" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E139" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F139" s="19" t="n"/>
+      <c r="G139" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="H139" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I139" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J139" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K139" s="19" t="n"/>
+      <c r="L139" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M139" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N139" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 80.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-14</t>
+        </is>
+      </c>
+      <c r="B140" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C140" s="19" t="inlineStr">
+        <is>
+          <t>CALF_RAISE</t>
+        </is>
+      </c>
+      <c r="D140" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="E140" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F140" s="19" t="n"/>
+      <c r="G140" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="H140" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I140" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J140" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K140" s="19" t="n"/>
+      <c r="L140" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M140" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N140" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 12 reps x 80.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-15</t>
+        </is>
+      </c>
+      <c r="B141" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C141" s="19" t="inlineStr">
+        <is>
+          <t>FLOOR_CRUNCH</t>
+        </is>
+      </c>
+      <c r="D141" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E141" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F141" s="19" t="n"/>
+      <c r="G141" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I141" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J141" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K141" s="19" t="n"/>
+      <c r="L141" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M141" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N141" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-16</t>
+        </is>
+      </c>
+      <c r="B142" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C142" s="19" t="inlineStr">
+        <is>
+          <t>FLOOR_CRUNCH</t>
+        </is>
+      </c>
+      <c r="D142" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E142" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F142" s="19" t="n"/>
+      <c r="G142" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I142" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J142" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K142" s="19" t="n"/>
+      <c r="L142" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M142" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N142" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-17</t>
+        </is>
+      </c>
+      <c r="B143" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C143" s="19" t="inlineStr">
+        <is>
+          <t>FLOOR_CRUNCH</t>
+        </is>
+      </c>
+      <c r="D143" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="E143" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F143" s="19" t="n"/>
+      <c r="G143" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I143" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J143" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K143" s="19" t="n"/>
+      <c r="L143" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M143" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N143" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-18</t>
+        </is>
+      </c>
+      <c r="B144" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C144" s="19" t="inlineStr">
+        <is>
+          <t>DEADBUG</t>
+        </is>
+      </c>
+      <c r="D144" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E144" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F144" s="19" t="n"/>
+      <c r="G144" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I144" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J144" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K144" s="19" t="n"/>
+      <c r="L144" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M144" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-19</t>
+        </is>
+      </c>
+      <c r="B145" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C145" s="19" t="inlineStr">
+        <is>
+          <t>DEADBUG</t>
+        </is>
+      </c>
+      <c r="D145" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="E145" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F145" s="19" t="n"/>
+      <c r="G145" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I145" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J145" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K145" s="19" t="n"/>
+      <c r="L145" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M145" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N145" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-20</t>
+        </is>
+      </c>
+      <c r="B146" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t>DEADBUG</t>
+        </is>
+      </c>
+      <c r="D146" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="E146" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F146" s="19" t="n"/>
+      <c r="G146" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I146" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J146" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K146" s="19" t="n"/>
+      <c r="L146" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M146" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="19" t="inlineStr">
+        <is>
+          <t>S-20261013-01-21</t>
+        </is>
+      </c>
+      <c r="B147" s="19" t="inlineStr">
+        <is>
+          <t>W-20261013-01</t>
+        </is>
+      </c>
+      <c r="C147" s="19" t="inlineStr">
+        <is>
+          <t>LYING_LEG_RAISE</t>
+        </is>
+      </c>
+      <c r="D147" s="19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E147" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F147" s="19" t="n"/>
+      <c r="G147" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I147" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J147" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K147" s="19" t="n"/>
+      <c r="L147" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M147" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N147" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 0.0 kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7762,7 +8922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -9160,6 +10320,96 @@
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>FLOOR_CRUNCH</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight Floor Crunch</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Obliques</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>bw_plus</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>LYING_LEG_RAISE</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Lying Leg Raise</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>Hip Flexors</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight</t>
+        </is>
+      </c>
+      <c r="F33" s="19" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>bw_plus</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>

</xml_diff>

<commit_message>
feat(workout): ingest Pull A session W-20261014-01 with straps breakthrough and update queue to Push B
</commit_message>
<xml_diff>
--- a/DASHBOARD/fitness_dashboard.xlsx
+++ b/DASHBOARD/fitness_dashboard.xlsx
@@ -780,8 +780,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H9" headerRowCount="1">
-  <autoFilter ref="A1:H9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H10" headerRowCount="1">
+  <autoFilter ref="A1:H10"/>
   <tableColumns count="8">
     <tableColumn id="1" name="workout_id"/>
     <tableColumn id="2" name="date"/>
@@ -797,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N147" headerRowCount="1">
-  <autoFilter ref="A1:N147"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N165" headerRowCount="1">
+  <autoFilter ref="A1:N165"/>
   <tableColumns count="14">
     <tableColumn id="1" name="set_id"/>
     <tableColumn id="2" name="workout_id"/>
@@ -820,8 +820,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I34" headerRowCount="1">
-  <autoFilter ref="A1:I34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I36" headerRowCount="1">
+  <autoFilter ref="A1:I36"/>
   <tableColumns count="9">
     <tableColumn id="1" name="exercise_id"/>
     <tableColumn id="2" name="exercise_name"/>
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1935,6 +1935,71 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Day 2: Pull A</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>68</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Workout
+2026-10-14 21:51
+Duration: 68m 4s
+Pull-up
+Set 1: 4 reps
+Set 2: 3 reps
+Lat Pulldown
+Set 1: 12 reps x 40.0 kg
+Set 2: 8 reps x 50.0 kg
+Set 3: 6 reps x 50.0 kg
+Machine Rear Delt Fly
+Set 1: 12 reps x 15.0 kg
+Set 2: 12 reps x 15.0 kg
+Set 3: 9 reps x 15.0 kg
+EZ Bar Curl
+Set 1: 15 reps x 20.0 kg
+Set 2: 12 reps x 20.0 kg
+Set 3: 11 reps x 20.0 kg
+Seated Row (Wide Grip)
+Set 1: 12 reps x 55.0 kg
+Set 2: 12 reps x 55.0 kg
+Set 3: 12 reps x 55.0 kg
+Hammer Curl
+Set 1: 12 reps x 5.0 kg
+Set 2: 10 reps x 7.5 kg
+Single Arm Lat Pulldown
+Set 1: 12 reps x 12.5 kg
+Set 2: 12 reps x 12.5 kg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1949,12 +2014,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N147"/>
+  <dimension ref="A1:N165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -8908,6 +8973,942 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-01</t>
+        </is>
+      </c>
+      <c r="B148" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t>PULL_UP</t>
+        </is>
+      </c>
+      <c r="D148" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F148" s="19" t="n"/>
+      <c r="G148" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I148" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J148" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K148" s="19" t="n"/>
+      <c r="L148" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M148" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N148" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 4 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-02</t>
+        </is>
+      </c>
+      <c r="B149" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C149" s="19" t="inlineStr">
+        <is>
+          <t>PULL_UP</t>
+        </is>
+      </c>
+      <c r="D149" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E149" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F149" s="19" t="n"/>
+      <c r="G149" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I149" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J149" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K149" s="19" t="n"/>
+      <c r="L149" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M149" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N149" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-03</t>
+        </is>
+      </c>
+      <c r="B150" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t>LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D150" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E150" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F150" s="19" t="n"/>
+      <c r="G150" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="H150" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I150" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J150" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K150" s="19" t="n"/>
+      <c r="L150" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M150" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N150" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 40.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-04</t>
+        </is>
+      </c>
+      <c r="B151" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C151" s="19" t="inlineStr">
+        <is>
+          <t>LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D151" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E151" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F151" s="19" t="n"/>
+      <c r="G151" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="H151" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I151" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J151" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K151" s="19" t="n"/>
+      <c r="L151" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M151" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N151" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 8 reps x 50.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-05</t>
+        </is>
+      </c>
+      <c r="B152" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C152" s="19" t="inlineStr">
+        <is>
+          <t>LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D152" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E152" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F152" s="19" t="n"/>
+      <c r="G152" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="H152" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I152" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J152" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K152" s="19" t="n"/>
+      <c r="L152" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M152" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N152" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 6 reps x 50.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-06</t>
+        </is>
+      </c>
+      <c r="B153" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C153" s="19" t="inlineStr">
+        <is>
+          <t>REAR_DELT_FLY</t>
+        </is>
+      </c>
+      <c r="D153" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E153" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F153" s="19" t="n"/>
+      <c r="G153" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H153" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I153" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J153" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K153" s="19" t="n"/>
+      <c r="L153" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M153" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N153" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 15.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-07</t>
+        </is>
+      </c>
+      <c r="B154" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C154" s="19" t="inlineStr">
+        <is>
+          <t>REAR_DELT_FLY</t>
+        </is>
+      </c>
+      <c r="D154" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E154" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F154" s="19" t="n"/>
+      <c r="G154" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H154" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I154" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J154" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K154" s="19" t="n"/>
+      <c r="L154" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M154" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 15.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-08</t>
+        </is>
+      </c>
+      <c r="B155" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C155" s="19" t="inlineStr">
+        <is>
+          <t>REAR_DELT_FLY</t>
+        </is>
+      </c>
+      <c r="D155" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E155" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F155" s="19" t="n"/>
+      <c r="G155" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H155" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I155" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="J155" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K155" s="19" t="n"/>
+      <c r="L155" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M155" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 9 reps x 15.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-09</t>
+        </is>
+      </c>
+      <c r="B156" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C156" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="D156" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E156" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F156" s="19" t="n"/>
+      <c r="G156" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H156" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I156" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="J156" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K156" s="19" t="n"/>
+      <c r="L156" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M156" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N156" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 15 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-10</t>
+        </is>
+      </c>
+      <c r="B157" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C157" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="D157" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E157" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F157" s="19" t="n"/>
+      <c r="G157" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H157" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I157" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J157" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K157" s="19" t="n"/>
+      <c r="L157" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M157" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N157" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-11</t>
+        </is>
+      </c>
+      <c r="B158" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C158" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="D158" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E158" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F158" s="19" t="n"/>
+      <c r="G158" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H158" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I158" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="J158" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K158" s="19" t="n"/>
+      <c r="L158" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M158" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N158" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 11 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-12</t>
+        </is>
+      </c>
+      <c r="B159" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C159" s="19" t="inlineStr">
+        <is>
+          <t>SEATED_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D159" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E159" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F159" s="19" t="n"/>
+      <c r="G159" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="H159" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I159" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J159" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K159" s="19" t="n"/>
+      <c r="L159" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M159" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N159" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 55.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-13</t>
+        </is>
+      </c>
+      <c r="B160" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C160" s="19" t="inlineStr">
+        <is>
+          <t>SEATED_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D160" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E160" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F160" s="19" t="n"/>
+      <c r="G160" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="H160" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I160" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J160" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K160" s="19" t="n"/>
+      <c r="L160" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M160" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 55.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-14</t>
+        </is>
+      </c>
+      <c r="B161" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C161" s="19" t="inlineStr">
+        <is>
+          <t>SEATED_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D161" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="E161" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F161" s="19" t="n"/>
+      <c r="G161" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="H161" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I161" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J161" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K161" s="19" t="n"/>
+      <c r="L161" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M161" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 12 reps x 55.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-15</t>
+        </is>
+      </c>
+      <c r="B162" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C162" s="19" t="inlineStr">
+        <is>
+          <t>HAMMER_CURL</t>
+        </is>
+      </c>
+      <c r="D162" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E162" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F162" s="19" t="n"/>
+      <c r="G162" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H162" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I162" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J162" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K162" s="19" t="n"/>
+      <c r="L162" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M162" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-16</t>
+        </is>
+      </c>
+      <c r="B163" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C163" s="19" t="inlineStr">
+        <is>
+          <t>HAMMER_CURL</t>
+        </is>
+      </c>
+      <c r="D163" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E163" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F163" s="19" t="n"/>
+      <c r="G163" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H163" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I163" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J163" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K163" s="19" t="n"/>
+      <c r="L163" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M163" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 10 reps x 7.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-17</t>
+        </is>
+      </c>
+      <c r="B164" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C164" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D164" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="E164" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F164" s="19" t="n"/>
+      <c r="G164" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H164" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I164" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J164" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K164" s="19" t="n"/>
+      <c r="L164" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M164" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 12.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="19" t="inlineStr">
+        <is>
+          <t>S-20261014-01-18</t>
+        </is>
+      </c>
+      <c r="B165" s="19" t="inlineStr">
+        <is>
+          <t>W-20261014-01</t>
+        </is>
+      </c>
+      <c r="C165" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D165" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E165" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F165" s="19" t="n"/>
+      <c r="G165" s="19" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H165" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I165" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J165" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K165" s="19" t="n"/>
+      <c r="L165" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M165" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 12.5 kg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -8922,10 +9923,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
@@ -10412,6 +11413,96 @@
       <c r="I33" s="19" t="inlineStr">
         <is>
           <t>Tier 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>EZ-Bar Bicep Curl</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Biceps</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>Brachialis</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Barbell</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>combined</t>
+        </is>
+      </c>
+      <c r="I34" s="19" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Single-Arm Cable Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>Lats</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Teres Major</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>Cable</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>machine_pin</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(workout): ingest Push B session W-20261016-01 with Pec Deck PR (+5kg) and advance queue to Pull B
</commit_message>
<xml_diff>
--- a/DASHBOARD/fitness_dashboard.xlsx
+++ b/DASHBOARD/fitness_dashboard.xlsx
@@ -780,8 +780,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H10" headerRowCount="1">
-  <autoFilter ref="A1:H10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H11" headerRowCount="1">
+  <autoFilter ref="A1:H11"/>
   <tableColumns count="8">
     <tableColumn id="1" name="workout_id"/>
     <tableColumn id="2" name="date"/>
@@ -797,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N165" headerRowCount="1">
-  <autoFilter ref="A1:N165"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N183" headerRowCount="1">
+  <autoFilter ref="A1:N183"/>
   <tableColumns count="14">
     <tableColumn id="1" name="set_id"/>
     <tableColumn id="2" name="workout_id"/>
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1560,7 +1560,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="595" customWidth="1" min="8" max="8"/>
+    <col width="815" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2000,6 +2000,71 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Day 5: Push B</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Workout
+2026-10-16 22:13
+Duration: 50m 54s
+Incline Dumbbell Press
+Set 1: 10 reps x 20.0 kg
+Set 2: 10 reps x 20.0 kg
+Set 3: 9 reps x 20.0 kg
+Overhead Tricep Extension
+Set 1: 10 reps x 15.0 kg
+Set 2: 10 reps x 15.0 kg
+Set 3: 10 reps x 15.0 kg
+Cable Lateral Raise
+Set 1: 12 reps x 2.5 kg
+Set 2: 12 reps x 2.5 kg
+Set 3: 16 reps x 2.5 kg
+Pec Deck Machine
+Set 1: 12 reps x 35.0 kg
+Set 2: 12 reps x 35.0 kg
+Set 3: 10 reps x 35.0 kg
+Dumbbell Lateral Raise
+Set 1: 12 reps x 5.0 kg
+Set 2: 12 reps x 5.0 kg
+Set 3 (dropset): 11 reps x 5.0 kg
+Set 4 (dropset): 14 reps x 2.5 kg
+Cable Tricep Pushdown
+Set 1: 12 reps x 20.0 kg
+Set 2: 13 reps x 20.0 kg
+Trainee Notes: did in order that is logged as machine was not availble for latral at that time switched to overhead so could do more i guess today for that as was not sore ..</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2014,7 +2079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N165"/>
+  <dimension ref="A1:N183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2030,7 +2095,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9906,6 +9971,946 @@
       <c r="N165" s="19" t="inlineStr">
         <is>
           <t>Set 2: 12 reps x 12.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-01</t>
+        </is>
+      </c>
+      <c r="B166" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C166" s="19" t="inlineStr">
+        <is>
+          <t>INCLINE_DB_PRESS</t>
+        </is>
+      </c>
+      <c r="D166" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E166" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F166" s="19" t="n"/>
+      <c r="G166" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H166" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I166" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J166" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K166" s="19" t="n"/>
+      <c r="L166" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M166" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 10 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-02</t>
+        </is>
+      </c>
+      <c r="B167" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C167" s="19" t="inlineStr">
+        <is>
+          <t>INCLINE_DB_PRESS</t>
+        </is>
+      </c>
+      <c r="D167" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E167" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F167" s="19" t="n"/>
+      <c r="G167" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H167" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I167" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J167" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K167" s="19" t="n"/>
+      <c r="L167" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M167" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N167" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 10 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-03</t>
+        </is>
+      </c>
+      <c r="B168" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C168" s="19" t="inlineStr">
+        <is>
+          <t>INCLINE_DB_PRESS</t>
+        </is>
+      </c>
+      <c r="D168" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F168" s="19" t="n"/>
+      <c r="G168" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H168" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I168" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="J168" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K168" s="19" t="n"/>
+      <c r="L168" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M168" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 9 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-04</t>
+        </is>
+      </c>
+      <c r="B169" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C169" s="19" t="inlineStr">
+        <is>
+          <t>OVERHEAD_TRICEPS_EXT</t>
+        </is>
+      </c>
+      <c r="D169" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E169" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F169" s="19" t="n"/>
+      <c r="G169" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H169" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I169" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J169" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K169" s="19" t="n"/>
+      <c r="L169" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M169" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 10 reps x 15.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-05</t>
+        </is>
+      </c>
+      <c r="B170" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C170" s="19" t="inlineStr">
+        <is>
+          <t>OVERHEAD_TRICEPS_EXT</t>
+        </is>
+      </c>
+      <c r="D170" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E170" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F170" s="19" t="n"/>
+      <c r="G170" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H170" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I170" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J170" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K170" s="19" t="n"/>
+      <c r="L170" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M170" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 10 reps x 15.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-06</t>
+        </is>
+      </c>
+      <c r="B171" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C171" s="19" t="inlineStr">
+        <is>
+          <t>OVERHEAD_TRICEPS_EXT</t>
+        </is>
+      </c>
+      <c r="D171" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E171" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F171" s="19" t="n"/>
+      <c r="G171" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H171" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I171" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J171" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K171" s="19" t="n"/>
+      <c r="L171" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M171" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 10 reps x 15.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-07</t>
+        </is>
+      </c>
+      <c r="B172" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C172" s="19" t="inlineStr">
+        <is>
+          <t>CABLE_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D172" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E172" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F172" s="19" t="n"/>
+      <c r="G172" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H172" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I172" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J172" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K172" s="19" t="n"/>
+      <c r="L172" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M172" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 2.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-08</t>
+        </is>
+      </c>
+      <c r="B173" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C173" s="19" t="inlineStr">
+        <is>
+          <t>CABLE_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D173" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E173" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F173" s="19" t="n"/>
+      <c r="G173" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H173" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I173" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J173" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K173" s="19" t="n"/>
+      <c r="L173" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M173" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N173" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 2.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-09</t>
+        </is>
+      </c>
+      <c r="B174" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C174" s="19" t="inlineStr">
+        <is>
+          <t>CABLE_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D174" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E174" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F174" s="19" t="n"/>
+      <c r="G174" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H174" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I174" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="J174" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K174" s="19" t="n"/>
+      <c r="L174" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M174" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N174" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 16 reps x 2.5 kg (Rep ceiling broken - load leap unlocked!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-10</t>
+        </is>
+      </c>
+      <c r="B175" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C175" s="19" t="inlineStr">
+        <is>
+          <t>PEC_DECK_FLY</t>
+        </is>
+      </c>
+      <c r="D175" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E175" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F175" s="19" t="n"/>
+      <c r="G175" s="19" t="n">
+        <v>35</v>
+      </c>
+      <c r="H175" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I175" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J175" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K175" s="19" t="n"/>
+      <c r="L175" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M175" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N175" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 35.0 kg (NEW LOAD PR +5kg!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-11</t>
+        </is>
+      </c>
+      <c r="B176" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C176" s="19" t="inlineStr">
+        <is>
+          <t>PEC_DECK_FLY</t>
+        </is>
+      </c>
+      <c r="D176" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E176" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F176" s="19" t="n"/>
+      <c r="G176" s="19" t="n">
+        <v>35</v>
+      </c>
+      <c r="H176" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I176" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J176" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K176" s="19" t="n"/>
+      <c r="L176" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M176" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N176" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 35.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-12</t>
+        </is>
+      </c>
+      <c r="B177" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C177" s="19" t="inlineStr">
+        <is>
+          <t>PEC_DECK_FLY</t>
+        </is>
+      </c>
+      <c r="D177" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E177" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F177" s="19" t="n"/>
+      <c r="G177" s="19" t="n">
+        <v>35</v>
+      </c>
+      <c r="H177" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I177" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J177" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K177" s="19" t="n"/>
+      <c r="L177" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M177" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N177" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 10 reps x 35.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-13</t>
+        </is>
+      </c>
+      <c r="B178" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C178" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D178" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E178" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F178" s="19" t="n"/>
+      <c r="G178" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H178" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I178" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J178" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K178" s="19" t="n"/>
+      <c r="L178" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M178" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N178" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-14</t>
+        </is>
+      </c>
+      <c r="B179" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C179" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D179" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="E179" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F179" s="19" t="n"/>
+      <c r="G179" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H179" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I179" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J179" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K179" s="19" t="n"/>
+      <c r="L179" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M179" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N179" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 12 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-15</t>
+        </is>
+      </c>
+      <c r="B180" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C180" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D180" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E180" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F180" s="19" t="n"/>
+      <c r="G180" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H180" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I180" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="J180" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K180" s="19" t="n"/>
+      <c r="L180" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M180" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N180" s="19" t="inlineStr">
+        <is>
+          <t>Set 3 (dropset parent): 11 reps x 5.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-16</t>
+        </is>
+      </c>
+      <c r="B181" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C181" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D181" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E181" s="19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F181" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-15</t>
+        </is>
+      </c>
+      <c r="G181" s="19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H181" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I181" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="J181" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K181" s="19" t="n"/>
+      <c r="L181" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M181" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N181" s="19" t="inlineStr">
+        <is>
+          <t>Set 4 (dropset): 14 reps x 2.5 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-17</t>
+        </is>
+      </c>
+      <c r="B182" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C182" s="19" t="inlineStr">
+        <is>
+          <t>TRICEPS_PUSHDOWN</t>
+        </is>
+      </c>
+      <c r="D182" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="E182" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F182" s="19" t="n"/>
+      <c r="G182" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H182" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I182" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J182" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K182" s="19" t="n"/>
+      <c r="L182" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="M182" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N182" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12 reps x 20.0 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="19" t="inlineStr">
+        <is>
+          <t>S-20261016-01-18</t>
+        </is>
+      </c>
+      <c r="B183" s="19" t="inlineStr">
+        <is>
+          <t>W-20261016-01</t>
+        </is>
+      </c>
+      <c r="C183" s="19" t="inlineStr">
+        <is>
+          <t>TRICEPS_PUSHDOWN</t>
+        </is>
+      </c>
+      <c r="D183" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E183" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F183" s="19" t="n"/>
+      <c r="G183" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H183" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I183" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="J183" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K183" s="19" t="n"/>
+      <c r="L183" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="M183" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N183" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 13 reps x 20.0 kg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ingest Oct 18 Pull B workout, update progress, advance queue to Push A
</commit_message>
<xml_diff>
--- a/DASHBOARD/fitness_dashboard.xlsx
+++ b/DASHBOARD/fitness_dashboard.xlsx
@@ -780,8 +780,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H11" headerRowCount="1">
-  <autoFilter ref="A1:H11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H12" headerRowCount="1">
+  <autoFilter ref="A1:H12"/>
   <tableColumns count="8">
     <tableColumn id="1" name="workout_id"/>
     <tableColumn id="2" name="date"/>
@@ -797,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N183" headerRowCount="1">
-  <autoFilter ref="A1:N183"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N205" headerRowCount="1">
+  <autoFilter ref="A1:N205"/>
   <tableColumns count="14">
     <tableColumn id="1" name="set_id"/>
     <tableColumn id="2" name="workout_id"/>
@@ -820,8 +820,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I36" headerRowCount="1">
-  <autoFilter ref="A1:I36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I37" headerRowCount="1">
+  <autoFilter ref="A1:I37"/>
   <tableColumns count="9">
     <tableColumn id="1" name="exercise_id"/>
     <tableColumn id="2" name="exercise_name"/>
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1560,7 +1560,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="815" customWidth="1" min="8" max="8"/>
+    <col width="1741" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2065,6 +2065,90 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Day 6: Pull B</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>101</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H12" s="19">
+        <f>== WORKOUT REPORT ===
+Pull b i guess not a but sending in pull a section as I can see pull b here in app
+Name:      Workout
+Date:      Sunday, Oct 18 2026 – 1:27 PM
+Duration:  101m 35s
+Volume:    5955.0 kg
+Sets:      22
+Exercises: 7
+--- Straight Arm Pulldown ---
+Set 1: 15.0 kg × 12 reps
+Set 2: 15.0 kg × 12 reps
+Set 3: 15.0 kg × 12 reps
+--- Close Grip Lat Pulldown ---
+Set 1: 45.0 kg × 10 reps
+Set 2: 45.0 kg × 8 reps
+Set 3: 40.0 kg × 8 reps
+--- Seated Row (V-Bar) ---
+Set 1: 60.0 kg × 12 reps
+Set 2: 65.0 kg × 12 reps
+Set 3: 65.0 kg × 9 reps
+--- Single Arm Cable Row ---
+Set 1: 12.0 kg × 10 reps
+Set 2: 15.0 kg × 15 reps
+Set 3: 20.0 kg × 12 reps
+Set 4: 15.0 kg × 12 reps
+--- Machine Rear Delt Fly ---
+Set 1: 15.0 kg × 12 reps
+Set 2: 15.0 kg × 12 reps
+Set 3: 15.0 kg × 12 reps
+--- EZ Bar Curl ---
+Set 1: 20.0 kg × 12 reps
+Set 2: 20.0 kg × 10 reps
+Set 3: 20.0 kg × 10 reps
+--- Hammer Curl ---
+Set 1: 5.0 kg × 12 reps
+Set 2: 7.5 kg × 15 reps [PR]
+Set 3: 7.5 kg × 11 reps
+--- XP ---
+Rear Delts: +54 XP
+Biceps: +118 XP
+Forearms: +58 XP
+Lats: +130 XP
+Upper Back: +82 XP
+Abs: +18 XP
+Total: +460 XP
+========================
+All went great except single arm lat now what bad in it idk... Felt or not felt MMC idk .. just felt kinda weird idk which muscle from I was pulling kinda all went tired and I was going and going in small can't pull in hard so took some time to find the weight suited for rep also I hard swing while seating make i shoulder a bit ouch not so much I think will be good next session ...
+But I need a proper guide to do this ex and to feel if I should continue a proper guide and how to feel it and do it ... Maybe not done that kuch so.. but idk you decide based on whatever my history this ex history reputation and all</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2079,7 +2163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N183"/>
+  <dimension ref="A1:N205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10914,6 +10998,1150 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-01</t>
+        </is>
+      </c>
+      <c r="B184" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C184" s="19" t="inlineStr">
+        <is>
+          <t>STRAIGHT_ARM_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D184" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E184" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F184" s="19" t="n"/>
+      <c r="G184" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H184" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I184" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J184" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K184" s="19" t="n"/>
+      <c r="L184" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M184" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N184" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-02</t>
+        </is>
+      </c>
+      <c r="B185" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C185" s="19" t="inlineStr">
+        <is>
+          <t>STRAIGHT_ARM_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D185" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E185" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F185" s="19" t="n"/>
+      <c r="G185" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H185" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I185" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J185" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K185" s="19" t="n"/>
+      <c r="L185" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M185" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N185" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-03</t>
+        </is>
+      </c>
+      <c r="B186" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C186" s="19" t="inlineStr">
+        <is>
+          <t>STRAIGHT_ARM_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D186" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E186" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F186" s="19" t="n"/>
+      <c r="G186" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H186" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I186" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J186" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K186" s="19" t="n"/>
+      <c r="L186" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M186" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N186" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-04</t>
+        </is>
+      </c>
+      <c r="B187" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C187" s="19" t="inlineStr">
+        <is>
+          <t>LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D187" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E187" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F187" s="19" t="n"/>
+      <c r="G187" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H187" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I187" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J187" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K187" s="19" t="n"/>
+      <c r="L187" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M187" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N187" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 45.0 kg × 10 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-05</t>
+        </is>
+      </c>
+      <c r="B188" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C188" s="19" t="inlineStr">
+        <is>
+          <t>LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D188" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E188" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F188" s="19" t="n"/>
+      <c r="G188" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="H188" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I188" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J188" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K188" s="19" t="n"/>
+      <c r="L188" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M188" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N188" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 45.0 kg × 8 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-06</t>
+        </is>
+      </c>
+      <c r="B189" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C189" s="19" t="inlineStr">
+        <is>
+          <t>LAT_PULLDOWN</t>
+        </is>
+      </c>
+      <c r="D189" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E189" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F189" s="19" t="n"/>
+      <c r="G189" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="H189" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I189" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J189" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K189" s="19" t="n"/>
+      <c r="L189" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M189" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N189" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 40.0 kg × 8 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-07</t>
+        </is>
+      </c>
+      <c r="B190" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C190" s="19" t="inlineStr">
+        <is>
+          <t>SEATED_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D190" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E190" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F190" s="19" t="n"/>
+      <c r="G190" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="H190" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I190" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J190" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K190" s="19" t="n"/>
+      <c r="L190" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M190" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N190" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 60.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-08</t>
+        </is>
+      </c>
+      <c r="B191" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C191" s="19" t="inlineStr">
+        <is>
+          <t>SEATED_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D191" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E191" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F191" s="19" t="n"/>
+      <c r="G191" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="H191" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I191" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J191" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K191" s="19" t="n"/>
+      <c r="L191" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M191" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N191" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 65.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-09</t>
+        </is>
+      </c>
+      <c r="B192" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C192" s="19" t="inlineStr">
+        <is>
+          <t>SEATED_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D192" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E192" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F192" s="19" t="n"/>
+      <c r="G192" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="H192" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I192" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="J192" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K192" s="19" t="n"/>
+      <c r="L192" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M192" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N192" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 65.0 kg × 9 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-10</t>
+        </is>
+      </c>
+      <c r="B193" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C193" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D193" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E193" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F193" s="19" t="n"/>
+      <c r="G193" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H193" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I193" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J193" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K193" s="19" t="n"/>
+      <c r="L193" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M193" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N193" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 12.0 kg × 10 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-11</t>
+        </is>
+      </c>
+      <c r="B194" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C194" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D194" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E194" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F194" s="19" t="n"/>
+      <c r="G194" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H194" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I194" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="J194" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K194" s="19" t="n"/>
+      <c r="L194" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M194" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N194" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 15.0 kg × 15 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-12</t>
+        </is>
+      </c>
+      <c r="B195" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C195" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D195" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E195" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F195" s="19" t="n"/>
+      <c r="G195" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H195" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I195" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J195" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K195" s="19" t="n"/>
+      <c r="L195" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M195" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N195" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 20.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-13</t>
+        </is>
+      </c>
+      <c r="B196" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C196" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="D196" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E196" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F196" s="19" t="n"/>
+      <c r="G196" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H196" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I196" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J196" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K196" s="19" t="n"/>
+      <c r="L196" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M196" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N196" s="19" t="inlineStr">
+        <is>
+          <t>Set 4: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-14</t>
+        </is>
+      </c>
+      <c r="B197" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C197" s="19" t="inlineStr">
+        <is>
+          <t>REAR_DELT_FLY</t>
+        </is>
+      </c>
+      <c r="D197" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="E197" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F197" s="19" t="n"/>
+      <c r="G197" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H197" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I197" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J197" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K197" s="19" t="n"/>
+      <c r="L197" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M197" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N197" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-15</t>
+        </is>
+      </c>
+      <c r="B198" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C198" s="19" t="inlineStr">
+        <is>
+          <t>REAR_DELT_FLY</t>
+        </is>
+      </c>
+      <c r="D198" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E198" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F198" s="19" t="n"/>
+      <c r="G198" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H198" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I198" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J198" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K198" s="19" t="n"/>
+      <c r="L198" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M198" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N198" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-16</t>
+        </is>
+      </c>
+      <c r="B199" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C199" s="19" t="inlineStr">
+        <is>
+          <t>REAR_DELT_FLY</t>
+        </is>
+      </c>
+      <c r="D199" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E199" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F199" s="19" t="n"/>
+      <c r="G199" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H199" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I199" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J199" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K199" s="19" t="n"/>
+      <c r="L199" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M199" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N199" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-17</t>
+        </is>
+      </c>
+      <c r="B200" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C200" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="D200" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="E200" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F200" s="19" t="n"/>
+      <c r="G200" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H200" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I200" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J200" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K200" s="19" t="n"/>
+      <c r="L200" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M200" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N200" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 20.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-18</t>
+        </is>
+      </c>
+      <c r="B201" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C201" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="D201" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E201" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F201" s="19" t="n"/>
+      <c r="G201" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H201" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I201" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J201" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K201" s="19" t="n"/>
+      <c r="L201" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M201" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N201" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 20.0 kg × 10 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-19</t>
+        </is>
+      </c>
+      <c r="B202" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C202" s="19" t="inlineStr">
+        <is>
+          <t>EZ_BAR_CURL</t>
+        </is>
+      </c>
+      <c r="D202" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="E202" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F202" s="19" t="n"/>
+      <c r="G202" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H202" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I202" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J202" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K202" s="19" t="n"/>
+      <c r="L202" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M202" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N202" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 20.0 kg × 10 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-20</t>
+        </is>
+      </c>
+      <c r="B203" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C203" s="19" t="inlineStr">
+        <is>
+          <t>HAMMER_CURL</t>
+        </is>
+      </c>
+      <c r="D203" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="E203" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F203" s="19" t="n"/>
+      <c r="G203" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H203" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I203" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J203" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K203" s="19" t="n"/>
+      <c r="L203" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M203" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N203" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 5.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-21</t>
+        </is>
+      </c>
+      <c r="B204" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C204" s="19" t="inlineStr">
+        <is>
+          <t>HAMMER_CURL</t>
+        </is>
+      </c>
+      <c r="D204" s="19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E204" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F204" s="19" t="n"/>
+      <c r="G204" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H204" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I204" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="J204" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K204" s="19" t="n"/>
+      <c r="L204" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M204" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N204" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 7.5 kg × 15 reps [PR]</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="19" t="inlineStr">
+        <is>
+          <t>S-20261018-01-22</t>
+        </is>
+      </c>
+      <c r="B205" s="19" t="inlineStr">
+        <is>
+          <t>W-20261018-01</t>
+        </is>
+      </c>
+      <c r="C205" s="19" t="inlineStr">
+        <is>
+          <t>HAMMER_CURL</t>
+        </is>
+      </c>
+      <c r="D205" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="E205" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F205" s="19" t="n"/>
+      <c r="G205" s="19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H205" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I205" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="J205" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K205" s="19" t="n"/>
+      <c r="L205" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M205" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N205" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 7.5 kg × 11 reps</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -10928,7 +12156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -12506,6 +13734,51 @@
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>SINGLE_ARM_CABLE_ROW</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Single-Arm Cable Row</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>Lats</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Upper Back, Biceps</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>Cable</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>machine_pin</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>

</xml_diff>

<commit_message>
Ingest Oct 19 Push A workout, calibrate gym equipment constraints, and advance queue to Day 2 Pull A
</commit_message>
<xml_diff>
--- a/DASHBOARD/fitness_dashboard.xlsx
+++ b/DASHBOARD/fitness_dashboard.xlsx
@@ -780,8 +780,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H12" headerRowCount="1">
-  <autoFilter ref="A1:H12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_Workouts" displayName="Table_Workouts" ref="A1:H13" headerRowCount="1">
+  <autoFilter ref="A1:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="workout_id"/>
     <tableColumn id="2" name="date"/>
@@ -797,8 +797,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N205" headerRowCount="1">
-  <autoFilter ref="A1:N205"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table_WorkoutSets" displayName="Table_WorkoutSets" ref="A1:N223" headerRowCount="1">
+  <autoFilter ref="A1:N223"/>
   <tableColumns count="14">
     <tableColumn id="1" name="set_id"/>
     <tableColumn id="2" name="workout_id"/>
@@ -820,8 +820,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I37" headerRowCount="1">
-  <autoFilter ref="A1:I37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table_ExerciseCatalog" displayName="Table_ExerciseCatalog" ref="A1:I38" headerRowCount="1">
+  <autoFilter ref="A1:I38"/>
   <tableColumns count="9">
     <tableColumn id="1" name="exercise_id"/>
     <tableColumn id="2" name="exercise_name"/>
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2149,6 +2149,85 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Day 5: Push B</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>75</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H13" s="19">
+        <f>== WORKOUT REPORT ===
+Name:      Workout
+Date:      Monday, Oct 19 2026 – 4:15 PM
+Duration:  75m 29s
+Volume:    3475.0 kg
+Sets:      18
+Exercises: 6
+--- Incline Dumbbell Press ---
+Set 1: 22.5 kg × 10 reps [PR]
+Set 2: 22.5 kg × 9 reps
+Set 3: 20.0 kg × 10 reps
+--- Smith Machine Bench Press ---
+Set 1: 42.5 kg × 8 reps
+Set 2: 47.5 kg × 6 reps
+Set 3: 42.5 kg × 7 reps
+--- Dumbbell Lateral Raise ---
+Set 1: 5.0 kg × 15 reps
+Set 2: 5.0 kg × 12 reps
+Set 3: 5.0 kg × 12 reps
+Set 4: 5.0 kg × 11 reps
+--- Pec Deck Machine ---
+Set 1: 35.0 kg × 11 reps
+Set 2: 35.0 kg × 6 reps
+Set 3: 30.0 kg × 6 reps
+--- Cable Tricep Pushdown ---
+Set 1: 20.0 kg × 12 reps
+Set 2: 20.0 kg × 12 reps
+--- Overhead Tricep Extension ---
+Set 1: 15.0 kg × 12 reps
+Set 2: 20.0 kg × 6 reps [PR]
+Set 3: 15.0 kg × 8 reps
+--- XP ---
+Upper Chest: +68 XP
+Lower Chest: +21 XP
+Front Delts: +29 XP
+Side Delts: +80 XP
+Triceps: +145 XP
+Middle Chest: +57 XP
+Total: +400 XP
+========================
+Don't have 2.5 increments on machine it's like 5 on forward so had to stay or puls t in some where u said +2.5. Also ykg dumble not available
+Also more time as got a friend in between so some talk
+Trainee Notes: Trainee feedback: All gym rope equipment machines have 2.5kg plates starting some, but eventually all have +5kg plate increments. Dumbbells also lack 6kg (rack has 1, 2, 3, 4, 5, 7, 8 kg). More time taken due to chatting with a friend.</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2163,7 +2242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N205"/>
+  <dimension ref="A1:N223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12142,6 +12221,942 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-01</t>
+        </is>
+      </c>
+      <c r="B206" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C206" s="19" t="inlineStr">
+        <is>
+          <t>INCLINE_DB_PRESS</t>
+        </is>
+      </c>
+      <c r="D206" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F206" s="19" t="n"/>
+      <c r="G206" s="19" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H206" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I206" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J206" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K206" s="19" t="n"/>
+      <c r="L206" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M206" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N206" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 22.5 kg × 10 reps [PR]</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-02</t>
+        </is>
+      </c>
+      <c r="B207" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C207" s="19" t="inlineStr">
+        <is>
+          <t>INCLINE_DB_PRESS</t>
+        </is>
+      </c>
+      <c r="D207" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E207" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F207" s="19" t="n"/>
+      <c r="G207" s="19" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H207" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I207" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="J207" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K207" s="19" t="n"/>
+      <c r="L207" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M207" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N207" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 22.5 kg × 9 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-03</t>
+        </is>
+      </c>
+      <c r="B208" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C208" s="19" t="inlineStr">
+        <is>
+          <t>INCLINE_DB_PRESS</t>
+        </is>
+      </c>
+      <c r="D208" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E208" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F208" s="19" t="n"/>
+      <c r="G208" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H208" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I208" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="J208" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K208" s="19" t="n"/>
+      <c r="L208" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M208" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N208" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 20.0 kg × 10 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-04</t>
+        </is>
+      </c>
+      <c r="B209" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C209" s="19" t="inlineStr">
+        <is>
+          <t>SMITH_BENCH</t>
+        </is>
+      </c>
+      <c r="D209" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E209" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F209" s="19" t="n"/>
+      <c r="G209" s="19" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H209" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I209" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J209" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K209" s="19" t="n"/>
+      <c r="L209" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M209" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N209" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 42.5 kg × 8 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-05</t>
+        </is>
+      </c>
+      <c r="B210" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C210" s="19" t="inlineStr">
+        <is>
+          <t>SMITH_BENCH</t>
+        </is>
+      </c>
+      <c r="D210" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E210" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F210" s="19" t="n"/>
+      <c r="G210" s="19" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="H210" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I210" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J210" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K210" s="19" t="n"/>
+      <c r="L210" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M210" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N210" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 47.5 kg × 6 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-06</t>
+        </is>
+      </c>
+      <c r="B211" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C211" s="19" t="inlineStr">
+        <is>
+          <t>SMITH_BENCH</t>
+        </is>
+      </c>
+      <c r="D211" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E211" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F211" s="19" t="n"/>
+      <c r="G211" s="19" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H211" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I211" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="J211" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K211" s="19" t="n"/>
+      <c r="L211" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M211" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N211" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 42.5 kg × 7 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-07</t>
+        </is>
+      </c>
+      <c r="B212" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C212" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D212" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E212" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F212" s="19" t="n"/>
+      <c r="G212" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H212" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I212" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="J212" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K212" s="19" t="n"/>
+      <c r="L212" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M212" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N212" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 5.0 kg × 15 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-08</t>
+        </is>
+      </c>
+      <c r="B213" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C213" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D213" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E213" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F213" s="19" t="n"/>
+      <c r="G213" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H213" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I213" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J213" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K213" s="19" t="n"/>
+      <c r="L213" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M213" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N213" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 5.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-09</t>
+        </is>
+      </c>
+      <c r="B214" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C214" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D214" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E214" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F214" s="19" t="n"/>
+      <c r="G214" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H214" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I214" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J214" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K214" s="19" t="n"/>
+      <c r="L214" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M214" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N214" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 5.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-10</t>
+        </is>
+      </c>
+      <c r="B215" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C215" s="19" t="inlineStr">
+        <is>
+          <t>DB_LATERAL_RAISE</t>
+        </is>
+      </c>
+      <c r="D215" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E215" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F215" s="19" t="n"/>
+      <c r="G215" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H215" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I215" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="J215" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K215" s="19" t="n"/>
+      <c r="L215" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M215" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N215" s="19" t="inlineStr">
+        <is>
+          <t>Set 4: 5.0 kg × 11 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-11</t>
+        </is>
+      </c>
+      <c r="B216" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C216" s="19" t="inlineStr">
+        <is>
+          <t>PEC_DECK_FLY</t>
+        </is>
+      </c>
+      <c r="D216" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E216" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F216" s="19" t="n"/>
+      <c r="G216" s="19" t="n">
+        <v>35</v>
+      </c>
+      <c r="H216" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I216" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="J216" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K216" s="19" t="n"/>
+      <c r="L216" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M216" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N216" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 35.0 kg × 11 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-12</t>
+        </is>
+      </c>
+      <c r="B217" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C217" s="19" t="inlineStr">
+        <is>
+          <t>PEC_DECK_FLY</t>
+        </is>
+      </c>
+      <c r="D217" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E217" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F217" s="19" t="n"/>
+      <c r="G217" s="19" t="n">
+        <v>35</v>
+      </c>
+      <c r="H217" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I217" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J217" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K217" s="19" t="n"/>
+      <c r="L217" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M217" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N217" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 35.0 kg × 6 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-13</t>
+        </is>
+      </c>
+      <c r="B218" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C218" s="19" t="inlineStr">
+        <is>
+          <t>PEC_DECK_FLY</t>
+        </is>
+      </c>
+      <c r="D218" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E218" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F218" s="19" t="n"/>
+      <c r="G218" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="H218" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I218" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J218" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K218" s="19" t="n"/>
+      <c r="L218" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M218" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N218" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 30.0 kg × 6 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-14</t>
+        </is>
+      </c>
+      <c r="B219" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C219" s="19" t="inlineStr">
+        <is>
+          <t>TRICEPS_PUSHDOWN</t>
+        </is>
+      </c>
+      <c r="D219" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="E219" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F219" s="19" t="n"/>
+      <c r="G219" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H219" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I219" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J219" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K219" s="19" t="n"/>
+      <c r="L219" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M219" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N219" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 20.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-15</t>
+        </is>
+      </c>
+      <c r="B220" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C220" s="19" t="inlineStr">
+        <is>
+          <t>TRICEPS_PUSHDOWN</t>
+        </is>
+      </c>
+      <c r="D220" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E220" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F220" s="19" t="n"/>
+      <c r="G220" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H220" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I220" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J220" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K220" s="19" t="n"/>
+      <c r="L220" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M220" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N220" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 20.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-16</t>
+        </is>
+      </c>
+      <c r="B221" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C221" s="19" t="inlineStr">
+        <is>
+          <t>OVERHEAD_TRICEPS_EXT</t>
+        </is>
+      </c>
+      <c r="D221" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E221" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F221" s="19" t="n"/>
+      <c r="G221" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H221" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I221" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="J221" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K221" s="19" t="n"/>
+      <c r="L221" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M221" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N221" s="19" t="inlineStr">
+        <is>
+          <t>Set 1: 15.0 kg × 12 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-17</t>
+        </is>
+      </c>
+      <c r="B222" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C222" s="19" t="inlineStr">
+        <is>
+          <t>OVERHEAD_TRICEPS_EXT</t>
+        </is>
+      </c>
+      <c r="D222" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="E222" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F222" s="19" t="n"/>
+      <c r="G222" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H222" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I222" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J222" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K222" s="19" t="n"/>
+      <c r="L222" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M222" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N222" s="19" t="inlineStr">
+        <is>
+          <t>Set 2: 20.0 kg × 6 reps [PR]</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="19" t="inlineStr">
+        <is>
+          <t>S-20261019-01-18</t>
+        </is>
+      </c>
+      <c r="B223" s="19" t="inlineStr">
+        <is>
+          <t>W-20261019-01</t>
+        </is>
+      </c>
+      <c r="C223" s="19" t="inlineStr">
+        <is>
+          <t>OVERHEAD_TRICEPS_EXT</t>
+        </is>
+      </c>
+      <c r="D223" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="E223" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F223" s="19" t="n"/>
+      <c r="G223" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="H223" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I223" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J223" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K223" s="19" t="n"/>
+      <c r="L223" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M223" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N223" s="19" t="inlineStr">
+        <is>
+          <t>Set 3: 15.0 kg × 8 reps</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -12156,7 +13171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -13781,6 +14796,51 @@
       <c r="I36" s="19" t="inlineStr">
         <is>
           <t>Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>SMITH_BENCH</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>Smith Machine Bench Press</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>Chest</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>Anterior Deltoids, Triceps</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>6-10</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>180</v>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
+        <is>
+          <t>combined</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
         </is>
       </c>
     </row>

</xml_diff>